<commit_message>
Add preseason results and schedule updates
</commit_message>
<xml_diff>
--- a/backend/data/matches.xlsx
+++ b/backend/data/matches.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경기일정" sheetId="1" r:id="R2361313150a34de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상세일정" sheetId="2" r:id="R30effe0e6dd74a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="플레이오프" sheetId="3" r:id="Rd3c7688597214aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="4" r:id="R216ad7e66b9949cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="경기일정" sheetId="1" r:id="Rff575d04080449e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="상세일정" sheetId="2" r:id="R3493097830574c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="플레이오프" sheetId="3" r:id="Rfd4e2b0cbecb4b84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="4" r:id="Rf5da05fa8b344492"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,7 +42,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -69,6 +69,16 @@
         <x:fgColor rgb="FFEEF2F7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="24">
     <x:border/>
@@ -241,7 +251,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="85">
+  <x:cellXfs count="100">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -383,6 +393,47 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -613,8 +664,9 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
@@ -627,231 +679,313 @@
       <x:c r="C1" s="12" t="str">
         <x:v>팀B</x:v>
       </x:c>
+      <x:c r="D1" s="88" t="str">
+        <x:v>경기구분</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
-      <x:c r="A2" s="31" t="n">
+      <x:c r="A2" s="97" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B2" s="98" t="str">
+        <x:v>이준석</x:v>
+      </x:c>
+      <x:c r="C2" s="99" t="str">
+        <x:v>서종원</x:v>
+      </x:c>
+      <x:c r="D2" s="98" t="str">
+        <x:v>프리시즌</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="90" t="n">
         <x:v>46270</x:v>
       </x:c>
-      <x:c r="B2" s="32" t="str">
+      <x:c r="B3" s="91" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C2" s="33" t="str">
+      <x:c r="C3" s="92" t="str">
         <x:v>이준석</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="31" t="n">
+      <x:c r="D3" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="90" t="n">
         <x:v>46270</x:v>
       </x:c>
-      <x:c r="B3" s="32" t="str">
+      <x:c r="B4" s="91" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C3" s="33" t="str">
+      <x:c r="C4" s="92" t="str">
         <x:v>이상</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" ht="22" customHeight="1">
-      <x:c r="A4" s="31" t="n">
+      <x:c r="D4" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="90" t="n">
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="B4" s="32" t="str">
+      <x:c r="B5" s="91" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C4" s="33" t="str">
+      <x:c r="C5" s="92" t="str">
         <x:v>문권기</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="22" customHeight="1">
-      <x:c r="A5" s="31" t="n">
+      <x:c r="D5" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="90" t="n">
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="B5" s="32" t="str">
+      <x:c r="B6" s="91" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C5" s="33" t="str">
+      <x:c r="C6" s="92" t="str">
         <x:v>이준석</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="22" customHeight="1">
-      <x:c r="A6" s="31" t="n">
+      <x:c r="D6" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="90" t="n">
         <x:v>46277</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="str">
+      <x:c r="B7" s="91" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C6" s="33" t="str">
+      <x:c r="C7" s="92" t="str">
         <x:v>이상</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="22" customHeight="1">
-      <x:c r="A7" s="31" t="n">
+      <x:c r="D7" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="90" t="n">
         <x:v>46277</x:v>
       </x:c>
-      <x:c r="B7" s="32" t="str">
+      <x:c r="B8" s="91" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C7" s="33" t="str">
+      <x:c r="C8" s="92" t="str">
         <x:v>서종원</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="22" customHeight="1">
-      <x:c r="A8" s="31" t="n">
+      <x:c r="D8" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="90" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="B8" s="32" t="str">
+      <x:c r="B9" s="91" t="str">
         <x:v>주은성</x:v>
       </x:c>
-      <x:c r="C8" s="33" t="str">
+      <x:c r="C9" s="92" t="str">
         <x:v>문권기</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="22" customHeight="1">
-      <x:c r="A9" s="31" t="n">
+      <x:c r="D9" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="90" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="B9" s="32" t="str">
+      <x:c r="B10" s="91" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C9" s="33" t="str">
+      <x:c r="C10" s="92" t="str">
         <x:v>이준석</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
-      <x:c r="A10" s="31" t="n">
+      <x:c r="D10" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="90" t="n">
         <x:v>46284</x:v>
       </x:c>
-      <x:c r="B10" s="32" t="str">
+      <x:c r="B11" s="91" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C10" s="33" t="str">
+      <x:c r="C11" s="92" t="str">
         <x:v>이준석</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="31" t="n">
+      <x:c r="D11" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="90" t="n">
         <x:v>46284</x:v>
       </x:c>
-      <x:c r="B11" s="32" t="str">
+      <x:c r="B12" s="91" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C11" s="33" t="str">
+      <x:c r="C12" s="92" t="str">
         <x:v>서종원</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="31" t="n">
+      <x:c r="D12" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="90" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="B12" s="32" t="str">
+      <x:c r="B13" s="91" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C12" s="33" t="str">
+      <x:c r="C13" s="92" t="str">
         <x:v>서종원</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="31" t="n">
+      <x:c r="D13" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="90" t="n">
         <x:v>46285</x:v>
       </x:c>
-      <x:c r="B13" s="32" t="str">
+      <x:c r="B14" s="91" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C13" s="33" t="str">
+      <x:c r="C14" s="92" t="str">
         <x:v>주은성</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="31" t="n">
+      <x:c r="D14" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="90" t="n">
         <x:v>46291</x:v>
       </x:c>
-      <x:c r="B14" s="32" t="str">
+      <x:c r="B15" s="91" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C14" s="33" t="str">
+      <x:c r="C15" s="92" t="str">
         <x:v>서종원</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="31" t="n">
+      <x:c r="D15" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="90" t="n">
         <x:v>46291</x:v>
       </x:c>
-      <x:c r="B15" s="32" t="str">
+      <x:c r="B16" s="91" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C15" s="33" t="str">
+      <x:c r="C16" s="92" t="str">
         <x:v>주은성</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="31" t="n">
+      <x:c r="D16" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="90" t="n">
         <x:v>46292</x:v>
       </x:c>
-      <x:c r="B16" s="32" t="str">
+      <x:c r="B17" s="91" t="str">
         <x:v>이상</x:v>
       </x:c>
-      <x:c r="C16" s="33" t="str">
+      <x:c r="C17" s="92" t="str">
         <x:v>문권기</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="22" customHeight="1">
-      <x:c r="A17" s="31" t="n">
+      <x:c r="D17" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="90" t="n">
         <x:v>46292</x:v>
       </x:c>
-      <x:c r="B17" s="32" t="str">
+      <x:c r="B18" s="91" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C17" s="33" t="str">
+      <x:c r="C18" s="92" t="str">
         <x:v>주은성</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="22" customHeight="1">
-      <x:c r="A18" s="31" t="n">
+      <x:c r="D18" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="90" t="n">
         <x:v>46298</x:v>
       </x:c>
-      <x:c r="B18" s="32" t="str">
+      <x:c r="B19" s="91" t="str">
         <x:v>문권기</x:v>
       </x:c>
-      <x:c r="C18" s="33" t="str">
+      <x:c r="C19" s="92" t="str">
         <x:v>주은성</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="31" t="n">
+      <x:c r="D19" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="90" t="n">
         <x:v>46298</x:v>
       </x:c>
-      <x:c r="B19" s="32" t="str">
+      <x:c r="B20" s="91" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C19" s="33" t="str">
+      <x:c r="C20" s="92" t="str">
         <x:v>이상</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="31" t="n">
+      <x:c r="D20" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="93" t="n">
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="B20" s="32" t="str">
+      <x:c r="B21" s="94" t="str">
         <x:v>이준석</x:v>
       </x:c>
-      <x:c r="C20" s="33" t="str">
+      <x:c r="C21" s="95" t="str">
         <x:v>문권기</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="22" customHeight="1">
-      <x:c r="A21" s="34" t="n">
+      <x:c r="D21" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="96" t="n">
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="B21" s="35" t="str">
+      <x:c r="B22" s="91" t="str">
         <x:v>서종원</x:v>
       </x:c>
-      <x:c r="C21" s="36" t="str">
+      <x:c r="C22" s="91" t="str">
         <x:v>이상</x:v>
       </x:c>
+      <x:c r="D22" s="91" t="str">
+        <x:v>정규리그</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="D2:D100">
+      <x:formula1>"정규리그,프리시즌"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae5357b7d8884381"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra460b03c12824c97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1419,7 +1553,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f86471096e247e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4a431e6c1024de7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>